<commit_message>
test: add chat util tests + v0.2.0 test cases + update progress
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="v0.1.0" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="v0.1.1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="汇总" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="v0.2.0" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -47,19 +48,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <color rgb="FFF0F0F5"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FFF0F0F5"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <name val="Arial"/>
       <charset val="134"/>
       <family val="2"/>
@@ -82,11 +70,22 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="FFF0F0F5"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F0F0F5"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00F0F0F5"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +109,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF16161E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E1E2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00252533"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="0016161E"/>
       </patternFill>
     </fill>
@@ -119,12 +133,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF2A2A3A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF2A2A3A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF2A2A3A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF2A2A3A"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -160,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -171,38 +200,47 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -646,7 +684,7 @@
           <t>Vite 启动</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>运行 npm run dev:vite</t>
         </is>
@@ -1882,11 +1920,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>跳过</t>
+          <t>通过</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>我不知道userdata在哪，我们现在还会有这个文件夹吗，不过持久化确实是实现了</t>
         </is>
@@ -2198,11 +2236,11 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>失败</t>
+          <t>通过</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
-      <c r="I10" s="9" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>只要点击会话，就算没有做任何操作，还是会更新到当前时间</t>
         </is>
@@ -2345,7 +2383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="7"/>
@@ -2389,68 +2427,656 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>v0.1.0</t>
         </is>
       </c>
-      <c r="B2" s="11">
-        <f>COUNTA(v0.1.0!A:A)-1</f>
+      <c r="B2" s="7">
+        <f>COUNTA('v0.1.0'!A:A)-1</f>
         <v/>
       </c>
-      <c r="C2" s="11">
-        <f>COUNTIF(v0.1.0!G:G,"通过")+COUNTIF(v0.1.0!G:G,"失败")+COUNTIF(v0.1.0!G:G,"跳过")</f>
+      <c r="C2" s="7">
+        <f>COUNTIF('v0.1.0'!G:G,"通过")+COUNTIF('v0.1.0'!G:G,"失败")+COUNTIF('v0.1.0'!G:G,"跳过")</f>
         <v/>
       </c>
-      <c r="D2" s="11">
-        <f>COUNTIF(v0.1.0!G:G,"通过")</f>
+      <c r="D2" s="7">
+        <f>COUNTIF('v0.1.0'!G:G,"通过")</f>
         <v/>
       </c>
-      <c r="E2" s="11">
-        <f>COUNTIF(v0.1.0!G:G,"失败")</f>
+      <c r="E2" s="7">
+        <f>COUNTIF('v0.1.0'!G:G,"失败")</f>
         <v/>
       </c>
-      <c r="F2" s="11">
-        <f>COUNTIF(v0.1.0!G:G,"跳过")</f>
+      <c r="F2" s="7">
+        <f>COUNTIF('v0.1.0'!G:G,"跳过")</f>
         <v/>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="11">
         <f>IF(C2&gt;0,D2/C2,0)</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>v0.1.1</t>
         </is>
       </c>
-      <c r="B3" s="13">
-        <f>COUNTA(v0.1.1!A:A)-1</f>
+      <c r="B3" s="9">
+        <f>COUNTA('v0.1.1'!A:A)-1</f>
         <v/>
       </c>
-      <c r="C3" s="13">
-        <f>COUNTIF(v0.1.1!G:G,"通过")+COUNTIF(v0.1.1!G:G,"失败")+COUNTIF(v0.1.1!G:G,"跳过")</f>
+      <c r="C3" s="9">
+        <f>COUNTIF('v0.1.1'!G:G,"通过")+COUNTIF('v0.1.1'!G:G,"失败")+COUNTIF('v0.1.1'!G:G,"跳过")</f>
         <v/>
       </c>
-      <c r="D3" s="13">
-        <f>COUNTIF(v0.1.1!G:G,"通过")</f>
+      <c r="D3" s="9">
+        <f>COUNTIF('v0.1.1'!G:G,"通过")</f>
         <v/>
       </c>
-      <c r="E3" s="13">
-        <f>COUNTIF(v0.1.1!G:G,"失败")</f>
+      <c r="E3" s="9">
+        <f>COUNTIF('v0.1.1'!G:G,"失败")</f>
         <v/>
       </c>
-      <c r="F3" s="13">
-        <f>COUNTIF(v0.1.1!G:G,"跳过")</f>
+      <c r="F3" s="9">
+        <f>COUNTIF('v0.1.1'!G:G,"跳过")</f>
         <v/>
       </c>
-      <c r="G3" s="14">
+      <c r="G3" s="12">
         <f>IF(C3&gt;0,D3/C3,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>v0.2.0</t>
+        </is>
+      </c>
+      <c r="B4" s="13">
+        <f>COUNTA(v0.2.0!A:A)-1</f>
+        <v/>
+      </c>
+      <c r="C4" s="13">
+        <f>COUNTIF(v0.2.0!G:G,"通过")+COUNTIF(v0.2.0!G:G,"失败")+COUNTIF(v0.2.0!G:G,"跳过")</f>
+        <v/>
+      </c>
+      <c r="D4" s="13">
+        <f>COUNTIF(v0.2.0!G:G,"通过")</f>
+        <v/>
+      </c>
+      <c r="E4" s="13">
+        <f>COUNTIF(v0.2.0!G:G,"失败")</f>
+        <v/>
+      </c>
+      <c r="F4" s="13">
+        <f>COUNTIF(v0.2.0!G:G,"跳过")</f>
+        <v/>
+      </c>
+      <c r="G4" s="14">
+        <f>IF(C4&gt;0,D4/C4,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007C6CFF"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>用例编号</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>模块</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>测试项</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>操作步骤</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>预期结果</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>实际结果</t>
+        </is>
+      </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>T-020-1</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>默认暗色主题</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>首次启动应用</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>显示暗色主题</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G2" s="16" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="16" t="inlineStr"/>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>T-020-2</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>切换亮色</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>设置→点击浅色</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>界面切换为亮色，过渡平滑</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H3" s="17" t="inlineStr"/>
+      <c r="I3" s="17" t="inlineStr"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>T-020-3</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>亮色持久化</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>切换亮色→重启</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>仍为亮色</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>未实现持久化</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>T-021-1</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>API配置</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>添加配置</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>设置→添加→填写→保存</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>列表出现新配置</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr"/>
+      <c r="I5" s="17" t="inlineStr"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>T-021-2</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>API配置</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>切换配置</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>点击不同配置</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>高亮切换</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr"/>
+      <c r="I6" s="16" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>T-021-3</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>API配置</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>删除配置</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>点击删除按钮</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>配置移除</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr"/>
+      <c r="I7" s="17" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>T-022-1</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>角色编辑</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>新建角色</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>侧边栏→角色→添加→编辑→保存</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>角色库出现新角色</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr"/>
+      <c r="I8" s="16" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>T-022-2</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>角色编辑</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>编辑角色</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>点击角色→修改字段→保存</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>角色信息更新</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr"/>
+      <c r="I9" s="17" t="inlineStr"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>T-022-3</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>角色编辑</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>加入会话</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>角色列表中点击加入会话</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>角色出现在右侧面板角色列表</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr"/>
+      <c r="I10" s="16" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>T-023-1</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>单角色对话</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>发送消息</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>角色加入会话→切换发言身份→发消息</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>AI 以角色身份回复</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr"/>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>需配置 API Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>T-023-2</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>单角色对话</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>流式输出</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>观察 AI 回复过程</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>文字逐字出现</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr"/>
+      <c r="I12" s="16" t="inlineStr"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>T-023-3</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>单角色对话</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>角色一致性</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>连续对话 5 轮</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>角色保持性格一致</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>待测试</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr"/>
+      <c r="I13" s="17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="F2:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="请选择 P0、P1 或 P2" type="list">
+      <formula1>"P0,P1,P2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="请选择有效状态" type="list">
+      <formula1>"待测试,通过,失败,跳过"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>